<commit_message>
Convert marketing spend workbook from INR millions to INR crores
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECbmyw4hK3nAiJnv9FLQpX
</commit_message>
<xml_diff>
--- a/outputs/Marketing_Spend_by_Bucket_FY24-FY26.xlsx
+++ b/outputs/Marketing_Spend_by_Bucket_FY24-FY26.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Marketing Spend by Bucket – FY24 to FY26 (Actuals)</t>
   </si>
   <si>
-    <t xml:space="preserve">INR in millions · Source: Finance advertisement expense sheet, mapped to buckets in "Line Item Mapping"</t>
+    <t xml:space="preserve">INR in crores (converted from finance sheet INR millions ÷ 10) · Source: Finance advertisement expense sheet, mapped to buckets in "Line Item Mapping"</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing bucket</t>
@@ -41,13 +41,13 @@
     <t xml:space="preserve">What it covers</t>
   </si>
   <si>
-    <t xml:space="preserve">FY24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY26</t>
+    <t xml:space="preserve">FY24 (₹ Cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25 (₹ Cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 (₹ Cr)</t>
   </si>
   <si>
     <t xml:space="preserve">FY24 mix %</t>
@@ -182,10 +182,10 @@
     <t xml:space="preserve">1. FY24–FY26 are actuals from the finance advertisement expense schedule (Management information). FY27 budget is not part of this data – see "FY27 Budget" tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. FY26 total here (415.52) ties to the finance schedule; finance notes a 0.25 difference vs. the audited FS figure (415.78).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. "Misc. / Unallocated" in FY26 includes a 3.83 unreconciled difference and a -2.07 reversal on unidentified vendor entries (per finance).</t>
+    <t xml:space="preserve">2. FY26 total here (41.55 Cr) ties to the finance schedule; finance notes a 0.03 Cr difference vs. the audited FS figure (41.58 Cr).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. "Misc. / Unallocated" in FY26 includes a 0.38 Cr unreconciled difference and a -0.21 Cr reversal on unidentified vendor entries (per finance).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Mapping of smaller vendors is inferred from vendor name – see confidence column in "Line Item Mapping". Change the bucket there and this summary updates.</t>
@@ -194,7 +194,7 @@
     <t xml:space="preserve">FY26 Marketing Spend – Bucket &gt; Activity breakdown</t>
   </si>
   <si>
-    <t xml:space="preserve">INR in millions · Line items with zero FY26 spend omitted</t>
+    <t xml:space="preserve">INR in crores (converted from finance sheet INR millions ÷ 10) · Line items with zero FY26 spend omitted</t>
   </si>
   <si>
     <t xml:space="preserve">Bucket / activity</t>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">Quarterly Ad Spend – Platform-level (FY24–FY26)</t>
   </si>
   <si>
-    <t xml:space="preserve">INR in millions · Quarterly split available from finance only for ad platforms &amp; vendor lines (not for SMS, branding, influencer, freebies, others)</t>
+    <t xml:space="preserve">INR in crores (converted from finance sheet INR millions ÷ 10) · Quarterly split available from finance only for ad platforms &amp; vendor lines (not for SMS, branding, influencer, freebies, others)</t>
   </si>
   <si>
     <t xml:space="preserve">Platform</t>
@@ -458,13 +458,13 @@
     <t xml:space="preserve">FY27 Marketing Budget by Bucket</t>
   </si>
   <si>
-    <t xml:space="preserve">INR in millions · Yellow cells to be filled by marketing (FY27 budget is not in the finance data shared)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY26 actual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FY27 budget</t>
+    <t xml:space="preserve">INR in crores (converted from finance sheet INR millions ÷ 10) · Yellow cells to be filled by marketing (FY27 budget is not in the finance data shared)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 actual (₹ Cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 budget (₹ Cr)</t>
   </si>
   <si>
     <t xml:space="preserve">Growth vs FY26</t>
@@ -476,13 +476,13 @@
     <t xml:space="preserve">Planned key activities</t>
   </si>
   <si>
-    <t xml:space="preserve">Example: Performance Marketing – D2C Website → FY27 budget 300.00, activities "Meta prospecting + retargeting, Google Search/PMax/Shopping".</t>
+    <t xml:space="preserve">Example: Performance Marketing – D2C Website → FY27 budget 30.00, activities "Meta prospecting + retargeting, Google Search/PMax/Shopping".</t>
   </si>
   <si>
     <t xml:space="preserve">Advertisement expense – line-item mapping to marketing buckets</t>
   </si>
   <si>
-    <t xml:space="preserve">INR in millions · Actuals · Source: Finance "Advertisement" sheet (Management information)</t>
+    <t xml:space="preserve">INR in crores (converted from finance sheet INR millions ÷ 10) · Actuals · Source: Finance "Advertisement" sheet (Management information)</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -1532,15 +1532,15 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A5)</f>
-        <v>129.98116253</v>
+        <v>12.998116253</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A5)</f>
-        <v>177.53210151</v>
+        <v>17.753210151</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A5)</f>
-        <v>248.3986606</v>
+        <v>24.83986606</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C5/C$16)</f>
@@ -1576,15 +1576,15 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A6)</f>
-        <v>17.1652215</v>
+        <v>1.71652215</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A6)</f>
-        <v>38.12716219</v>
+        <v>3.812716219</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A6)</f>
-        <v>120.45059929</v>
+        <v>12.045059929</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C6/C$16)</f>
@@ -1624,11 +1624,11 @@
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A7)</f>
-        <v>2.15</v>
+        <v>0.215</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A7)</f>
-        <v>8.5448946</v>
+        <v>0.85448946</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C7/C$16)</f>
@@ -1664,15 +1664,15 @@
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A8)</f>
-        <v>11.39013377</v>
+        <v>1.139013377</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A8)</f>
-        <v>7.97322871</v>
+        <v>0.797322871</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A8)</f>
-        <v>8.18497047</v>
+        <v>0.818497047</v>
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C8/C$16)</f>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="J8" s="7" t="n">
         <f aca="false">IF(D8=0,"n.m.",E8/D8-1)</f>
-        <v>0.0265565892690918</v>
+        <v>0.0265565892690915</v>
       </c>
       <c r="K8" s="7" t="n">
         <f aca="false">IF($E$18=0,0,E8/$E$18)</f>
@@ -1708,15 +1708,15 @@
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A9)</f>
-        <v>1.21511931</v>
+        <v>0.121511931</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A9)</f>
-        <v>1.0658553</v>
+        <v>0.10658553</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A9)</f>
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="F9" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C9/C$16)</f>
@@ -1752,15 +1752,15 @@
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A10)</f>
-        <v>3.14826724</v>
+        <v>0.314826724</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A10)</f>
-        <v>3.98518829</v>
+        <v>0.398518829</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A10)</f>
-        <v>11.16663002</v>
+        <v>1.116663002</v>
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C10/C$16)</f>
@@ -1796,15 +1796,15 @@
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A11)</f>
-        <v>0.763441</v>
+        <v>0.0763441</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A11)</f>
-        <v>15.464863</v>
+        <v>1.5464863</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A11)</f>
-        <v>10.77239666</v>
+        <v>1.077239666</v>
       </c>
       <c r="F11" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C11/C$16)</f>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="H11" s="7" t="n">
         <f aca="false">IF(E$16=0,0,E11/E$16)</f>
-        <v>0.02592492017787</v>
+        <v>0.0259249201778701</v>
       </c>
       <c r="I11" s="7" t="n">
         <f aca="false">IF(C11=0,"n.m.",D11/C11-1)</f>
@@ -1824,11 +1824,11 @@
       </c>
       <c r="J11" s="7" t="n">
         <f aca="false">IF(D11=0,"n.m.",E11/D11-1)</f>
-        <v>-0.303427604887286</v>
+        <v>-0.303427604887285</v>
       </c>
       <c r="K11" s="7" t="n">
         <f aca="false">IF($E$18=0,0,E11/$E$18)</f>
-        <v>0.00523627595571475</v>
+        <v>0.00523627595571476</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1840,15 +1840,15 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A12)</f>
-        <v>0.38568508</v>
+        <v>0.038568508</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A12)</f>
-        <v>0.98795763</v>
+        <v>0.098795763</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A12)</f>
-        <v>3.794468</v>
+        <v>0.3794468</v>
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C12/C$16)</f>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">IF(E$16=0,0,E12/E$16)</f>
-        <v>0.00913179147800543</v>
+        <v>0.00913179147800544</v>
       </c>
       <c r="I12" s="7" t="n">
         <f aca="false">IF(C12=0,"n.m.",D12/C12-1)</f>
@@ -1884,15 +1884,15 @@
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A13)</f>
-        <v>17.839522</v>
+        <v>1.7839522</v>
       </c>
       <c r="D13" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A13)</f>
-        <v>9.19406226</v>
+        <v>0.919406226</v>
       </c>
       <c r="E13" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A13)</f>
-        <v>1.37142119</v>
+        <v>0.137142119</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C13/C$16)</f>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="I13" s="7" t="n">
         <f aca="false">IF(C13=0,"n.m.",D13/C13-1)</f>
-        <v>-0.484623956852655</v>
+        <v>-0.484623956852656</v>
       </c>
       <c r="J13" s="7" t="n">
         <f aca="false">IF(D13=0,"n.m.",E13/D13-1)</f>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="K13" s="7" t="n">
         <f aca="false">IF($E$18=0,0,E13/$E$18)</f>
-        <v>0.000666624153287975</v>
+        <v>0.000666624153287976</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1928,15 +1928,15 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A14)</f>
-        <v>0.1815665</v>
+        <v>0.01815665</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A14)</f>
-        <v>0.28092792</v>
+        <v>0.028092792</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A14)</f>
-        <v>0.30403944</v>
+        <v>0.030403944</v>
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C14/C$16)</f>
@@ -1972,15 +1972,15 @@
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$F$5:$F$77,'Line Item Mapping'!$C$5:$C$77,$A15)</f>
-        <v>2.26548510999999</v>
+        <v>0.226548510999999</v>
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$G$5:$G$77,'Line Item Mapping'!$C$5:$C$77,$A15)</f>
-        <v>3.12296</v>
+        <v>0.312296</v>
       </c>
       <c r="E15" s="6" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,$A15)</f>
-        <v>2.33476748000011</v>
+        <v>0.233476748000011</v>
       </c>
       <c r="F15" s="7" t="n">
         <f aca="false">IF(C$16=0,0,C15/C$16)</f>
@@ -2014,15 +2014,15 @@
       <c r="B16" s="8"/>
       <c r="C16" s="9" t="n">
         <f aca="false">SUM(C5:C15)</f>
-        <v>184.33560404</v>
+        <v>18.433560404</v>
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">SUM(D5:D15)</f>
-        <v>259.88430681</v>
+        <v>25.988430681</v>
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">SUM(E5:E15)</f>
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
       <c r="F16" s="10" t="n">
         <f aca="false">SUM(F5:F15)</f>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="I16" s="10" t="n">
         <f aca="false">D16/C16-1</f>
-        <v>0.4098432484785</v>
+        <v>0.409843248478499</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">E16/D16-1</f>
@@ -2057,13 +2057,13 @@
         <v>37</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>843.81490685</v>
+        <v>84.381490685</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1102.82116883</v>
+        <v>110.282116883</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>2057.2629768</v>
+        <v>205.72629768</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2117,15 +2117,15 @@
       </c>
       <c r="C24" s="18" t="n">
         <f aca="false">C5+C6+C7+C8+C9</f>
-        <v>159.75163711</v>
+        <v>15.975163711</v>
       </c>
       <c r="D24" s="18" t="n">
         <f aca="false">D5+D6+D7+D8+D9</f>
-        <v>226.84834771</v>
+        <v>22.684834771</v>
       </c>
       <c r="E24" s="18" t="n">
         <f aca="false">E5+E6+E7+E8+E9</f>
-        <v>385.77912496</v>
+        <v>38.577912496</v>
       </c>
       <c r="F24" s="19" t="n">
         <f aca="false">E24/$E$16</f>
@@ -2141,15 +2141,15 @@
       </c>
       <c r="C25" s="18" t="n">
         <f aca="false">C11+C12+C13</f>
-        <v>18.98864808</v>
+        <v>1.898864808</v>
       </c>
       <c r="D25" s="18" t="n">
         <f aca="false">D11+D12+D13</f>
-        <v>25.64688289</v>
+        <v>2.564688289</v>
       </c>
       <c r="E25" s="18" t="n">
         <f aca="false">E11+E12+E13</f>
-        <v>15.93828585</v>
+        <v>1.593828585</v>
       </c>
       <c r="F25" s="19" t="n">
         <f aca="false">E25/$E$16</f>
@@ -2165,15 +2165,15 @@
       </c>
       <c r="C26" s="18" t="n">
         <f aca="false">C10+C14+C15</f>
-        <v>5.59531884999999</v>
+        <v>0.559531884999999</v>
       </c>
       <c r="D26" s="18" t="n">
         <f aca="false">D10+D14+D15</f>
-        <v>7.38907621</v>
+        <v>0.738907621</v>
       </c>
       <c r="E26" s="18" t="n">
         <f aca="false">E10+E14+E15</f>
-        <v>13.8054369400001</v>
+        <v>1.38054369400001</v>
       </c>
       <c r="F26" s="19" t="n">
         <f aca="false">E26/$E$16</f>
@@ -2187,15 +2187,15 @@
       <c r="B27" s="20"/>
       <c r="C27" s="9" t="n">
         <f aca="false">SUM(C24:C26)</f>
-        <v>184.33560404</v>
+        <v>18.433560404</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">SUM(D24:D26)</f>
-        <v>259.88430681</v>
+        <v>25.988430681</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">SUM(E24:E26)</f>
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
       <c r="F27" s="10" t="n">
         <f aca="false">SUM(F24:F26)</f>
@@ -2286,7 +2286,7 @@
       <c r="B5" s="8"/>
       <c r="C5" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A5)</f>
-        <v>248.3986606</v>
+        <v>24.83986606</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="10" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H5</f>
-        <v>198.11683608</v>
+        <v>19.811683608</v>
       </c>
       <c r="D6" s="26" t="n">
         <f aca="false">IF($C$5=0,0,C6/$C$5)</f>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H6</f>
-        <v>50.28182452</v>
+        <v>5.028182452</v>
       </c>
       <c r="D7" s="26" t="n">
         <f aca="false">IF($C$5=0,0,C7/$C$5)</f>
@@ -2341,7 +2341,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A8)</f>
-        <v>120.45059929</v>
+        <v>12.045059929</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="10" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H7</f>
-        <v>107.03484217</v>
+        <v>10.703484217</v>
       </c>
       <c r="D9" s="26" t="n">
         <f aca="false">IF($C$8=0,0,C9/$C$8)</f>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="C10" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H8</f>
-        <v>7.82607124</v>
+        <v>0.782607124</v>
       </c>
       <c r="D10" s="26" t="n">
         <f aca="false">IF($C$8=0,0,C10/$C$8)</f>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="C11" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H9</f>
-        <v>3.29217816</v>
+        <v>0.329217816</v>
       </c>
       <c r="D11" s="26" t="n">
         <f aca="false">IF($C$8=0,0,C11/$C$8)</f>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="C12" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H10</f>
-        <v>2.29750772</v>
+        <v>0.229750772</v>
       </c>
       <c r="D12" s="26" t="n">
         <f aca="false">IF($C$8=0,0,C12/$C$8)</f>
@@ -2436,7 +2436,7 @@
       <c r="B13" s="8"/>
       <c r="C13" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A13)</f>
-        <v>8.5448946</v>
+        <v>0.85448946</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="10" t="n">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="C14" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H11</f>
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="D14" s="26" t="n">
         <f aca="false">IF($C$13=0,0,C14/$C$13)</f>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="C15" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H12</f>
-        <v>1.1081856</v>
+        <v>0.11081856</v>
       </c>
       <c r="D15" s="26" t="n">
         <f aca="false">IF($C$13=0,0,C15/$C$13)</f>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C16" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H13</f>
-        <v>0.436709</v>
+        <v>0.0436709</v>
       </c>
       <c r="D16" s="26" t="n">
         <f aca="false">IF($C$13=0,0,C16/$C$13)</f>
@@ -2511,7 +2511,7 @@
       <c r="B17" s="8"/>
       <c r="C17" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A17)</f>
-        <v>8.18497047</v>
+        <v>0.818497047</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="10" t="n">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="C18" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H14</f>
-        <v>7.9997</v>
+        <v>0.79997</v>
       </c>
       <c r="D18" s="26" t="n">
         <f aca="false">IF($C$17=0,0,C18/$C$17)</f>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="C19" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H16</f>
-        <v>0.11027047</v>
+        <v>0.011027047</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">IF($C$17=0,0,C19/$C$17)</f>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="C20" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H15</f>
-        <v>0.075</v>
+        <v>0.0075</v>
       </c>
       <c r="D20" s="26" t="n">
         <f aca="false">IF($C$17=0,0,C20/$C$17)</f>
@@ -2586,7 +2586,7 @@
       <c r="B21" s="8"/>
       <c r="C21" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A21)</f>
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="10" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="C22" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H24</f>
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="D22" s="26" t="n">
         <f aca="false">IF($C$21=0,0,C22/$C$21)</f>
@@ -2621,7 +2621,7 @@
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A23)</f>
-        <v>11.16663002</v>
+        <v>1.116663002</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="10" t="n">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C24" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H39</f>
-        <v>8.91663002</v>
+        <v>0.891663002</v>
       </c>
       <c r="D24" s="26" t="n">
         <f aca="false">IF($C$23=0,0,C24/$C$23)</f>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="C25" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H38</f>
-        <v>2.25</v>
+        <v>0.225</v>
       </c>
       <c r="D25" s="26" t="n">
         <f aca="false">IF($C$23=0,0,C25/$C$23)</f>
@@ -2676,12 +2676,12 @@
       <c r="B26" s="8"/>
       <c r="C26" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A26)</f>
-        <v>10.77239666</v>
+        <v>1.077239666</v>
       </c>
       <c r="D26" s="8"/>
       <c r="E26" s="10" t="n">
         <f aca="false">C26/$C$49</f>
-        <v>0.02592492017787</v>
+        <v>0.0259249201778701</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="C27" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H49</f>
-        <v>5.20763666</v>
+        <v>0.520763666</v>
       </c>
       <c r="D27" s="26" t="n">
         <f aca="false">IF($C$26=0,0,C27/$C$26)</f>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="C28" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H50</f>
-        <v>2.78976</v>
+        <v>0.278976</v>
       </c>
       <c r="D28" s="26" t="n">
         <f aca="false">IF($C$26=0,0,C28/$C$26)</f>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C29" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H51</f>
-        <v>1.555</v>
+        <v>0.1555</v>
       </c>
       <c r="D29" s="26" t="n">
         <f aca="false">IF($C$26=0,0,C29/$C$26)</f>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="C30" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H40</f>
-        <v>0.9</v>
+        <v>0.09</v>
       </c>
       <c r="D30" s="26" t="n">
         <f aca="false">IF($C$26=0,0,C30/$C$26)</f>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C31" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H41</f>
-        <v>0.32</v>
+        <v>0.032</v>
       </c>
       <c r="D31" s="26" t="n">
         <f aca="false">IF($C$26=0,0,C31/$C$26)</f>
@@ -2791,12 +2791,12 @@
       <c r="B32" s="8"/>
       <c r="C32" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A32)</f>
-        <v>3.794468</v>
+        <v>0.3794468</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="10" t="n">
         <f aca="false">C32/$C$49</f>
-        <v>0.00913179147800543</v>
+        <v>0.00913179147800544</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C33" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H63</f>
-        <v>3.50192</v>
+        <v>0.350192</v>
       </c>
       <c r="D33" s="26" t="n">
         <f aca="false">IF($C$32=0,0,C33/$C$32)</f>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="C34" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H52</f>
-        <v>0.202548</v>
+        <v>0.0202548</v>
       </c>
       <c r="D34" s="26" t="n">
         <f aca="false">IF($C$32=0,0,C34/$C$32)</f>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="C35" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H53</f>
-        <v>0.09</v>
+        <v>0.009</v>
       </c>
       <c r="D35" s="26" t="n">
         <f aca="false">IF($C$32=0,0,C35/$C$32)</f>
@@ -2866,7 +2866,7 @@
       <c r="B36" s="8"/>
       <c r="C36" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A36)</f>
-        <v>1.37142119</v>
+        <v>0.137142119</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="10" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C37" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H65</f>
-        <v>1.37142119</v>
+        <v>0.137142119</v>
       </c>
       <c r="D37" s="26" t="n">
         <f aca="false">IF($C$36=0,0,C37/$C$36)</f>
@@ -2901,7 +2901,7 @@
       <c r="B38" s="8"/>
       <c r="C38" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A38)</f>
-        <v>0.30403944</v>
+        <v>0.030403944</v>
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="10" t="n">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="C39" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H71</f>
-        <v>0.148</v>
+        <v>0.0148</v>
       </c>
       <c r="D39" s="26" t="n">
         <f aca="false">IF($C$38=0,0,C39/$C$38)</f>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="C40" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H66</f>
-        <v>0.1196</v>
+        <v>0.01196</v>
       </c>
       <c r="D40" s="26" t="n">
         <f aca="false">IF($C$38=0,0,C40/$C$38)</f>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="C41" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H67</f>
-        <v>0.0211</v>
+        <v>0.00211</v>
       </c>
       <c r="D41" s="26" t="n">
         <f aca="false">IF($C$38=0,0,C41/$C$38)</f>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="C42" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H68</f>
-        <v>0.01533944</v>
+        <v>0.001533944</v>
       </c>
       <c r="D42" s="26" t="n">
         <f aca="false">IF($C$38=0,0,C42/$C$38)</f>
@@ -2996,7 +2996,7 @@
       <c r="B43" s="8"/>
       <c r="C43" s="9" t="n">
         <f aca="false">SUMIFS('Line Item Mapping'!$H$5:$H$77,'Line Item Mapping'!$C$5:$C$77,A43)</f>
-        <v>2.33476748000011</v>
+        <v>0.233476748000011</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="10" t="n">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C44" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H77</f>
-        <v>3.83262019000011</v>
+        <v>0.383262019000011</v>
       </c>
       <c r="D44" s="26" t="n">
         <f aca="false">IF($C$43=0,0,C44/$C$43)</f>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C45" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H72</f>
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="D45" s="26" t="n">
         <f aca="false">IF($C$43=0,0,C45/$C$43)</f>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="C46" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H73</f>
-        <v>0.2123802</v>
+        <v>0.02123802</v>
       </c>
       <c r="D46" s="26" t="n">
         <f aca="false">IF($C$43=0,0,C46/$C$43)</f>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C47" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H75</f>
-        <v>0.06333509</v>
+        <v>0.006333509</v>
       </c>
       <c r="D47" s="26" t="n">
         <f aca="false">IF($C$43=0,0,C47/$C$43)</f>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C48" s="25" t="n">
         <f aca="false">'Line Item Mapping'!H74</f>
-        <v>-2.073568</v>
+        <v>-0.2073568</v>
       </c>
       <c r="D48" s="26" t="n">
         <f aca="false">IF($C$43=0,0,C48/$C$43)</f>
@@ -3111,7 +3111,7 @@
       <c r="B49" s="8"/>
       <c r="C49" s="9" t="n">
         <f aca="false">C5+C8+C13+C17+C21+C23+C26+C32+C36+C38+C43</f>
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="10" t="n">
@@ -3204,51 +3204,51 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">SUM(B6:B7)</f>
-        <v>29.76424991</v>
+        <v>2.976424991</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">SUM(C6:C7)</f>
-        <v>30.55136732</v>
+        <v>3.055136732</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">SUM(D6:D7)</f>
-        <v>33.65355905</v>
+        <v>3.365355905</v>
       </c>
       <c r="E5" s="9" t="n">
         <f aca="false">SUM(E6:E7)</f>
-        <v>36.01198625</v>
+        <v>3.601198625</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">SUM(F6:F7)</f>
-        <v>37.07579475</v>
+        <v>3.707579475</v>
       </c>
       <c r="G5" s="9" t="n">
         <f aca="false">SUM(G6:G7)</f>
-        <v>42.58839042</v>
+        <v>4.258839042</v>
       </c>
       <c r="H5" s="9" t="n">
         <f aca="false">SUM(H6:H7)</f>
-        <v>46.11955595</v>
+        <v>4.611955595</v>
       </c>
       <c r="I5" s="9" t="n">
         <f aca="false">SUM(I6:I7)</f>
-        <v>51.74836039</v>
+        <v>5.174836039</v>
       </c>
       <c r="J5" s="9" t="n">
         <f aca="false">SUM(J6:J7)</f>
-        <v>51.9595885</v>
+        <v>5.19595885</v>
       </c>
       <c r="K5" s="9" t="n">
         <f aca="false">SUM(K6:K7)</f>
-        <v>58.52287808</v>
+        <v>5.852287808</v>
       </c>
       <c r="L5" s="9" t="n">
         <f aca="false">SUM(L6:L7)</f>
-        <v>60.52968029</v>
+        <v>6.052968029</v>
       </c>
       <c r="M5" s="9" t="n">
         <f aca="false">SUM(M6:M7)</f>
-        <v>77.38651373</v>
+        <v>7.738651373</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3256,40 +3256,40 @@
         <v>60</v>
       </c>
       <c r="B6" s="27" t="n">
-        <v>18.98788296</v>
+        <v>1.898788296</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>20.90611013</v>
+        <v>2.090611013</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>22.49599158</v>
+        <v>2.249599158</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>26.00002043</v>
+        <v>2.600002043</v>
       </c>
       <c r="F6" s="27" t="n">
-        <v>26.96075943</v>
+        <v>2.696075943</v>
       </c>
       <c r="G6" s="27" t="n">
-        <v>32.29524154</v>
+        <v>3.229524154</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>34.19861544</v>
+        <v>3.419861544</v>
       </c>
       <c r="I6" s="27" t="n">
-        <v>39.11840547</v>
+        <v>3.911840547</v>
       </c>
       <c r="J6" s="27" t="n">
-        <v>39.6840459</v>
+        <v>3.96840459</v>
       </c>
       <c r="K6" s="27" t="n">
-        <v>45.75812202</v>
+        <v>4.575812202</v>
       </c>
       <c r="L6" s="27" t="n">
-        <v>49.32136609</v>
+        <v>4.932136609</v>
       </c>
       <c r="M6" s="27" t="n">
-        <v>63.35330207</v>
+        <v>6.335330207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3297,40 +3297,40 @@
         <v>62</v>
       </c>
       <c r="B7" s="27" t="n">
-        <v>10.77636695</v>
+        <v>1.077636695</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>9.64525719</v>
+        <v>0.964525719</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>11.15756747</v>
+        <v>1.115756747</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>10.01196582</v>
+        <v>1.001196582</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>10.11503532</v>
+        <v>1.011503532</v>
       </c>
       <c r="G7" s="27" t="n">
-        <v>10.29314888</v>
+        <v>1.029314888</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>11.92094051</v>
+        <v>1.192094051</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>12.62995492</v>
+        <v>1.262995492</v>
       </c>
       <c r="J7" s="27" t="n">
-        <v>12.2755426</v>
+        <v>1.22755426</v>
       </c>
       <c r="K7" s="27" t="n">
-        <v>12.76475606</v>
+        <v>1.276475606</v>
       </c>
       <c r="L7" s="27" t="n">
-        <v>11.2083142</v>
+        <v>1.12083142</v>
       </c>
       <c r="M7" s="27" t="n">
-        <v>14.03321166</v>
+        <v>1.403321166</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3339,51 +3339,51 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">SUM(B9:B12)</f>
-        <v>6.7648045</v>
+        <v>0.67648045</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">SUM(C9:C12)</f>
-        <v>4.30217149</v>
+        <v>0.430217149</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">SUM(D9:D12)</f>
-        <v>3.35064309</v>
+        <v>0.335064309</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">SUM(E9:E12)</f>
-        <v>2.74760242</v>
+        <v>0.274760242</v>
       </c>
       <c r="F8" s="9" t="n">
         <f aca="false">SUM(F9:F12)</f>
-        <v>4.29050277</v>
+        <v>0.429050277</v>
       </c>
       <c r="G8" s="9" t="n">
         <f aca="false">SUM(G9:G12)</f>
-        <v>10.70139385</v>
+        <v>1.070139385</v>
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">SUM(H9:H12)</f>
-        <v>9.48261521</v>
+        <v>0.948261521</v>
       </c>
       <c r="I8" s="9" t="n">
         <f aca="false">SUM(I9:I12)</f>
-        <v>13.65265036</v>
+        <v>1.365265036</v>
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">SUM(J9:J12)</f>
-        <v>21.59556962</v>
+        <v>2.159556962</v>
       </c>
       <c r="K8" s="9" t="n">
         <f aca="false">SUM(K9:K12)</f>
-        <v>30.25863896</v>
+        <v>3.025863896</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">SUM(L9:L12)</f>
-        <v>32.14120573</v>
+        <v>3.214120573</v>
       </c>
       <c r="M8" s="9" t="n">
         <f aca="false">SUM(M9:M12)</f>
-        <v>36.45518498</v>
+        <v>3.645518498</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3391,40 +3391,40 @@
         <v>64</v>
       </c>
       <c r="B9" s="27" t="n">
-        <v>5.62563755</v>
+        <v>0.562563755</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>3.27814661</v>
+        <v>0.327814661</v>
       </c>
       <c r="D9" s="27" t="n">
-        <v>2.11661867</v>
+        <v>0.211661867</v>
       </c>
       <c r="E9" s="27" t="n">
-        <v>1.93698759</v>
+        <v>0.193698759</v>
       </c>
       <c r="F9" s="27" t="n">
-        <v>3.7177635</v>
+        <v>0.37177635</v>
       </c>
       <c r="G9" s="27" t="n">
-        <v>9.69156828</v>
+        <v>0.969156828</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>8.38307268</v>
+        <v>0.838307268</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>12.76976776</v>
+        <v>1.276976776</v>
       </c>
       <c r="J9" s="27" t="n">
-        <v>19.12698977</v>
+        <v>1.912698977</v>
       </c>
       <c r="K9" s="27" t="n">
-        <v>27.580355</v>
+        <v>2.7580355</v>
       </c>
       <c r="L9" s="27" t="n">
-        <v>28.62294634</v>
+        <v>2.862294634</v>
       </c>
       <c r="M9" s="27" t="n">
-        <v>31.70455106</v>
+        <v>3.170455106</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3456,16 +3456,16 @@
         <v>0</v>
       </c>
       <c r="J10" s="27" t="n">
-        <v>1.19189087</v>
+        <v>0.119189087</v>
       </c>
       <c r="K10" s="27" t="n">
-        <v>1.40236937</v>
+        <v>0.140236937</v>
       </c>
       <c r="L10" s="27" t="n">
-        <v>2.31441745</v>
+        <v>0.231441745</v>
       </c>
       <c r="M10" s="27" t="n">
-        <v>2.91739355</v>
+        <v>0.291739355</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,40 +3473,40 @@
         <v>68</v>
       </c>
       <c r="B11" s="27" t="n">
-        <v>0.42918395</v>
+        <v>0.042918395</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>0.66647388</v>
+        <v>0.066647388</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>1.04116142</v>
+        <v>0.104116142</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>0.51030483</v>
+        <v>0.051030483</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>0.34378027</v>
+        <v>0.034378027</v>
       </c>
       <c r="G11" s="27" t="n">
-        <v>0.68410457</v>
+        <v>0.068410457</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>0.67627553</v>
+        <v>0.067627553</v>
       </c>
       <c r="I11" s="27" t="n">
-        <v>0.4742286</v>
+        <v>0.04742286</v>
       </c>
       <c r="J11" s="27" t="n">
-        <v>0.91896898</v>
+        <v>0.091896898</v>
       </c>
       <c r="K11" s="27" t="n">
-        <v>1.05603359</v>
+        <v>0.105603359</v>
       </c>
       <c r="L11" s="27" t="n">
-        <v>1.12454594</v>
+        <v>0.112454594</v>
       </c>
       <c r="M11" s="27" t="n">
-        <v>0.19262965</v>
+        <v>0.019262965</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3514,40 +3514,40 @@
         <v>70</v>
       </c>
       <c r="B12" s="27" t="n">
-        <v>0.709983</v>
+        <v>0.0709983</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>0.357551</v>
+        <v>0.0357551</v>
       </c>
       <c r="D12" s="27" t="n">
-        <v>0.192863</v>
+        <v>0.0192863</v>
       </c>
       <c r="E12" s="27" t="n">
-        <v>0.30031</v>
+        <v>0.030031</v>
       </c>
       <c r="F12" s="27" t="n">
-        <v>0.228959</v>
+        <v>0.0228959</v>
       </c>
       <c r="G12" s="27" t="n">
-        <v>0.325721</v>
+        <v>0.0325721</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>0.423267</v>
+        <v>0.0423267</v>
       </c>
       <c r="I12" s="27" t="n">
-        <v>0.408654</v>
+        <v>0.0408654</v>
       </c>
       <c r="J12" s="27" t="n">
-        <v>0.35772</v>
+        <v>0.035772</v>
       </c>
       <c r="K12" s="27" t="n">
-        <v>0.219881</v>
+        <v>0.0219881</v>
       </c>
       <c r="L12" s="27" t="n">
-        <v>0.079296</v>
+        <v>0.0079296</v>
       </c>
       <c r="M12" s="27" t="n">
-        <v>1.64061072</v>
+        <v>0.164061072</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3584,23 +3584,23 @@
       </c>
       <c r="I13" s="9" t="n">
         <f aca="false">SUM(I14:I16)</f>
-        <v>2.15</v>
+        <v>0.215</v>
       </c>
       <c r="J13" s="9" t="n">
         <f aca="false">SUM(J14:J16)</f>
-        <v>0.1831856</v>
+        <v>0.01831856</v>
       </c>
       <c r="K13" s="9" t="n">
         <f aca="false">SUM(K14:K16)</f>
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="L13" s="9" t="n">
         <f aca="false">SUM(L14:L16)</f>
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M13" s="9" t="n">
         <f aca="false">SUM(M14:M16)</f>
-        <v>4.961709</v>
+        <v>0.4961709</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3635,13 +3635,13 @@
         <v>0</v>
       </c>
       <c r="K14" s="27" t="n">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="L14" s="27" t="n">
-        <v>2.6</v>
+        <v>0.26</v>
       </c>
       <c r="M14" s="27" t="n">
-        <v>4.1</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,19 +3670,19 @@
         <v>0</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>2.15</v>
+        <v>0.215</v>
       </c>
       <c r="J15" s="27" t="n">
-        <v>0.1831856</v>
+        <v>0.01831856</v>
       </c>
       <c r="K15" s="27" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="27" t="n">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="M15" s="27" t="n">
-        <v>0.425</v>
+        <v>0.0425</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3723,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="27" t="n">
-        <v>0.436709</v>
+        <v>0.0436709</v>
       </c>
     </row>
   </sheetData>
@@ -3762,7 +3762,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
         <v>2</v>
       </c>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">'Bucket Summary'!E5</f>
-        <v>248.3986606</v>
+        <v>24.83986606</v>
       </c>
       <c r="C5" s="30"/>
       <c r="D5" s="19" t="str">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="B6" s="29" t="n">
         <f aca="false">'Bucket Summary'!E6</f>
-        <v>120.45059929</v>
+        <v>12.045059929</v>
       </c>
       <c r="C6" s="30"/>
       <c r="D6" s="19" t="str">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">'Bucket Summary'!E7</f>
-        <v>8.5448946</v>
+        <v>0.85448946</v>
       </c>
       <c r="C7" s="30"/>
       <c r="D7" s="19" t="str">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="B8" s="29" t="n">
         <f aca="false">'Bucket Summary'!E8</f>
-        <v>8.18497047</v>
+        <v>0.818497047</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="19" t="str">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">'Bucket Summary'!E9</f>
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="19" t="str">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="B10" s="29" t="n">
         <f aca="false">'Bucket Summary'!E10</f>
-        <v>11.16663002</v>
+        <v>1.116663002</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="19" t="str">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="B11" s="29" t="n">
         <f aca="false">'Bucket Summary'!E11</f>
-        <v>10.77239666</v>
+        <v>1.077239666</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="19" t="str">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B12" s="29" t="n">
         <f aca="false">'Bucket Summary'!E12</f>
-        <v>3.794468</v>
+        <v>0.3794468</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="19" t="str">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="B13" s="29" t="n">
         <f aca="false">'Bucket Summary'!E13</f>
-        <v>1.37142119</v>
+        <v>0.137142119</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="19" t="str">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B14" s="29" t="n">
         <f aca="false">'Bucket Summary'!E14</f>
-        <v>0.30403944</v>
+        <v>0.030403944</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="19" t="str">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="B15" s="29" t="n">
         <f aca="false">'Bucket Summary'!E15</f>
-        <v>2.33476748000011</v>
+        <v>0.233476748000011</v>
       </c>
       <c r="C15" s="30"/>
       <c r="D15" s="19" t="str">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">SUM(C5:C15)</f>
@@ -4095,13 +4095,13 @@
         <v>157</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>88.3900051</v>
+        <v>8.83900051</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>132.57302188</v>
+        <v>13.257302188</v>
       </c>
       <c r="H5" s="33" t="n">
-        <v>198.11683608</v>
+        <v>19.811683608</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4121,13 +4121,13 @@
         <v>157</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>41.59115743</v>
+        <v>4.159115743</v>
       </c>
       <c r="G6" s="33" t="n">
-        <v>44.95907963</v>
+        <v>4.495907963</v>
       </c>
       <c r="H6" s="33" t="n">
-        <v>50.28182452</v>
+        <v>5.028182452</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4147,13 +4147,13 @@
         <v>157</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>12.95739042</v>
+        <v>1.295739042</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>34.56217222</v>
+        <v>3.456217222</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>107.03484217</v>
+        <v>10.703484217</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4179,7 +4179,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="33" t="n">
-        <v>7.82607124</v>
+        <v>0.782607124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4199,13 +4199,13 @@
         <v>157</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>2.64712408</v>
+        <v>0.264712408</v>
       </c>
       <c r="G9" s="33" t="n">
-        <v>2.17838897</v>
+        <v>0.217838897</v>
       </c>
       <c r="H9" s="33" t="n">
-        <v>3.29217816</v>
+        <v>0.329217816</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4225,13 +4225,13 @@
         <v>157</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>1.560707</v>
+        <v>0.1560707</v>
       </c>
       <c r="G10" s="33" t="n">
-        <v>1.386601</v>
+        <v>0.1386601</v>
       </c>
       <c r="H10" s="33" t="n">
-        <v>2.29750772</v>
+        <v>0.229750772</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4257,7 +4257,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>7</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4280,10 +4280,10 @@
         <v>0</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>2.15</v>
+        <v>0.215</v>
       </c>
       <c r="H12" s="33" t="n">
-        <v>1.1081856</v>
+        <v>0.11081856</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4309,7 +4309,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>0.436709</v>
+        <v>0.0436709</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4329,13 +4329,13 @@
         <v>157</v>
       </c>
       <c r="F14" s="33" t="n">
-        <v>7.64075411</v>
+        <v>0.764075411</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>6.56221316</v>
+        <v>0.656221316</v>
       </c>
       <c r="H14" s="33" t="n">
-        <v>7.9997</v>
+        <v>0.79997</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4361,7 +4361,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="33" t="n">
-        <v>0.075</v>
+        <v>0.0075</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4384,10 +4384,10 @@
         <v>0</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>0.16758311</v>
+        <v>0.016758311</v>
       </c>
       <c r="H16" s="33" t="n">
-        <v>0.11027047</v>
+        <v>0.011027047</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4410,7 +4410,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>0.010256</v>
+        <v>0.0010256</v>
       </c>
       <c r="H17" s="33" t="n">
         <v>0</v>
@@ -4433,7 +4433,7 @@
         <v>172</v>
       </c>
       <c r="F18" s="33" t="n">
-        <v>0.02305347</v>
+        <v>0.002305347</v>
       </c>
       <c r="G18" s="33" t="n">
         <v>0</v>
@@ -4459,7 +4459,7 @@
         <v>168</v>
       </c>
       <c r="F19" s="33" t="n">
-        <v>0.005</v>
+        <v>0.0005</v>
       </c>
       <c r="G19" s="33" t="n">
         <v>0</v>
@@ -4485,7 +4485,7 @@
         <v>172</v>
       </c>
       <c r="F20" s="33" t="n">
-        <v>0.00294938</v>
+        <v>0.000294938</v>
       </c>
       <c r="G20" s="33" t="n">
         <v>0</v>
@@ -4511,10 +4511,10 @@
         <v>172</v>
       </c>
       <c r="F21" s="33" t="n">
-        <v>0.06637681</v>
+        <v>0.006637681</v>
       </c>
       <c r="G21" s="33" t="n">
-        <v>0.029989</v>
+        <v>0.0029989</v>
       </c>
       <c r="H21" s="33" t="n">
         <v>0</v>
@@ -4537,10 +4537,10 @@
         <v>172</v>
       </c>
       <c r="F22" s="33" t="n">
-        <v>3.652</v>
+        <v>0.3652</v>
       </c>
       <c r="G22" s="33" t="n">
-        <v>1.197249</v>
+        <v>0.1197249</v>
       </c>
       <c r="H22" s="33" t="n">
         <v>0</v>
@@ -4566,7 +4566,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>0.00593844</v>
+        <v>0.000593844</v>
       </c>
       <c r="H23" s="33" t="n">
         <v>0</v>
@@ -4595,7 +4595,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4618,7 +4618,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="33" t="n">
-        <v>0.118</v>
+        <v>0.0118</v>
       </c>
       <c r="H25" s="33" t="n">
         <v>0</v>
@@ -4641,7 +4641,7 @@
         <v>168</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>0.17758396</v>
+        <v>0.017758396</v>
       </c>
       <c r="G26" s="33" t="n">
         <v>0</v>
@@ -4667,7 +4667,7 @@
         <v>157</v>
       </c>
       <c r="F27" s="33" t="n">
-        <v>0.04192945</v>
+        <v>0.004192945</v>
       </c>
       <c r="G27" s="33" t="n">
         <v>0</v>
@@ -4696,7 +4696,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="33" t="n">
-        <v>0.12711864</v>
+        <v>0.012711864</v>
       </c>
       <c r="H28" s="33" t="n">
         <v>0</v>
@@ -4719,10 +4719,10 @@
         <v>172</v>
       </c>
       <c r="F29" s="33" t="n">
-        <v>0.19589101</v>
+        <v>0.019589101</v>
       </c>
       <c r="G29" s="33" t="n">
-        <v>0.00259889</v>
+        <v>0.000259889</v>
       </c>
       <c r="H29" s="33" t="n">
         <v>0</v>
@@ -4745,7 +4745,7 @@
         <v>168</v>
       </c>
       <c r="F30" s="33" t="n">
-        <v>0.001544</v>
+        <v>0.0001544</v>
       </c>
       <c r="G30" s="33" t="n">
         <v>0</v>
@@ -4774,7 +4774,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="33" t="n">
-        <v>0.001716</v>
+        <v>0.0001716</v>
       </c>
       <c r="H31" s="33" t="n">
         <v>0</v>
@@ -4797,10 +4797,10 @@
         <v>172</v>
       </c>
       <c r="F32" s="33" t="n">
-        <v>0.01341285</v>
+        <v>0.001341285</v>
       </c>
       <c r="G32" s="33" t="n">
-        <v>0.00862158</v>
+        <v>0.000862158</v>
       </c>
       <c r="H32" s="33" t="n">
         <v>0</v>
@@ -4826,7 +4826,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="33" t="n">
-        <v>0.45</v>
+        <v>0.045</v>
       </c>
       <c r="H33" s="33" t="n">
         <v>0</v>
@@ -4849,10 +4849,10 @@
         <v>157</v>
       </c>
       <c r="F34" s="33" t="n">
-        <v>0.0081</v>
+        <v>0.00081</v>
       </c>
       <c r="G34" s="33" t="n">
-        <v>0.0039</v>
+        <v>0.00039</v>
       </c>
       <c r="H34" s="33" t="n">
         <v>0</v>
@@ -4875,10 +4875,10 @@
         <v>157</v>
       </c>
       <c r="F35" s="33" t="n">
-        <v>0.77665804</v>
+        <v>0.077665804</v>
       </c>
       <c r="G35" s="33" t="n">
-        <v>0.35390019</v>
+        <v>0.035390019</v>
       </c>
       <c r="H35" s="33" t="n">
         <v>0</v>
@@ -4901,10 +4901,10 @@
         <v>157</v>
       </c>
       <c r="F36" s="33" t="n">
-        <v>1.597769</v>
+        <v>0.1597769</v>
       </c>
       <c r="G36" s="33" t="n">
-        <v>1.90853975</v>
+        <v>0.190853975</v>
       </c>
       <c r="H36" s="33" t="n">
         <v>0</v>
@@ -4927,7 +4927,7 @@
         <v>157</v>
       </c>
       <c r="F37" s="33" t="n">
-        <v>6.96E-006</v>
+        <v>6.96E-007</v>
       </c>
       <c r="G37" s="33" t="n">
         <v>0</v>
@@ -4956,10 +4956,10 @@
         <v>0</v>
       </c>
       <c r="G38" s="33" t="n">
-        <v>0.861</v>
+        <v>0.0861</v>
       </c>
       <c r="H38" s="33" t="n">
-        <v>2.25</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4979,13 +4979,13 @@
         <v>157</v>
       </c>
       <c r="F39" s="33" t="n">
-        <v>1.55049128</v>
+        <v>0.155049128</v>
       </c>
       <c r="G39" s="33" t="n">
-        <v>1.21564854</v>
+        <v>0.121564854</v>
       </c>
       <c r="H39" s="33" t="n">
-        <v>8.91663002</v>
+        <v>0.891663002</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5011,7 +5011,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="33" t="n">
-        <v>0.9</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="33" t="n">
-        <v>0.32</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5060,7 +5060,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>3.7</v>
+        <v>0.37</v>
       </c>
       <c r="H42" s="33" t="n">
         <v>0</v>
@@ -5083,7 +5083,7 @@
         <v>172</v>
       </c>
       <c r="F43" s="33" t="n">
-        <v>0.075</v>
+        <v>0.0075</v>
       </c>
       <c r="G43" s="33" t="n">
         <v>0</v>
@@ -5109,7 +5109,7 @@
         <v>172</v>
       </c>
       <c r="F44" s="33" t="n">
-        <v>0.054</v>
+        <v>0.0054</v>
       </c>
       <c r="G44" s="33" t="n">
         <v>0</v>
@@ -5135,7 +5135,7 @@
         <v>172</v>
       </c>
       <c r="F45" s="33" t="n">
-        <v>0.03159</v>
+        <v>0.003159</v>
       </c>
       <c r="G45" s="33" t="n">
         <v>0</v>
@@ -5164,7 +5164,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>1.104301</v>
+        <v>0.1104301</v>
       </c>
       <c r="H46" s="33" t="n">
         <v>0</v>
@@ -5190,7 +5190,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="33" t="n">
-        <v>2.2265</v>
+        <v>0.22265</v>
       </c>
       <c r="H47" s="33" t="n">
         <v>0</v>
@@ -5216,7 +5216,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="33" t="n">
-        <v>4.08</v>
+        <v>0.408</v>
       </c>
       <c r="H48" s="33" t="n">
         <v>0</v>
@@ -5245,7 +5245,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="33" t="n">
-        <v>5.20763666</v>
+        <v>0.520763666</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5265,13 +5265,13 @@
         <v>157</v>
       </c>
       <c r="F50" s="33" t="n">
-        <v>0.602851</v>
+        <v>0.0602851</v>
       </c>
       <c r="G50" s="33" t="n">
-        <v>4.354062</v>
+        <v>0.4354062</v>
       </c>
       <c r="H50" s="33" t="n">
-        <v>2.78976</v>
+        <v>0.278976</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5297,7 +5297,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="33" t="n">
-        <v>1.555</v>
+        <v>0.1555</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5323,7 +5323,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="33" t="n">
-        <v>0.202548</v>
+        <v>0.0202548</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5346,10 +5346,10 @@
         <v>0</v>
       </c>
       <c r="G53" s="33" t="n">
-        <v>0.09</v>
+        <v>0.009</v>
       </c>
       <c r="H53" s="33" t="n">
-        <v>0.09</v>
+        <v>0.009</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5372,7 +5372,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="33" t="n">
-        <v>0.002</v>
+        <v>0.0002</v>
       </c>
       <c r="H54" s="33" t="n">
         <v>0</v>
@@ -5398,7 +5398,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="33" t="n">
-        <v>0.015</v>
+        <v>0.0015</v>
       </c>
       <c r="H55" s="33" t="n">
         <v>0</v>
@@ -5421,7 +5421,7 @@
         <v>168</v>
       </c>
       <c r="F56" s="33" t="n">
-        <v>0.00026825</v>
+        <v>2.6825E-005</v>
       </c>
       <c r="G56" s="33" t="n">
         <v>0</v>
@@ -5447,7 +5447,7 @@
         <v>168</v>
       </c>
       <c r="F57" s="33" t="n">
-        <v>0.02</v>
+        <v>0.002</v>
       </c>
       <c r="G57" s="33" t="n">
         <v>0</v>
@@ -5473,7 +5473,7 @@
         <v>172</v>
       </c>
       <c r="F58" s="33" t="n">
-        <v>0.03821683</v>
+        <v>0.003821683</v>
       </c>
       <c r="G58" s="33" t="n">
         <v>0</v>
@@ -5502,7 +5502,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="33" t="n">
-        <v>0.0335</v>
+        <v>0.00335</v>
       </c>
       <c r="H59" s="33" t="n">
         <v>0</v>
@@ -5525,7 +5525,7 @@
         <v>172</v>
       </c>
       <c r="F60" s="33" t="n">
-        <v>0.02</v>
+        <v>0.002</v>
       </c>
       <c r="G60" s="33" t="n">
         <v>0</v>
@@ -5551,7 +5551,7 @@
         <v>172</v>
       </c>
       <c r="F61" s="33" t="n">
-        <v>0.015</v>
+        <v>0.0015</v>
       </c>
       <c r="G61" s="33" t="n">
         <v>0</v>
@@ -5580,7 +5580,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="33" t="n">
-        <v>0.84745763</v>
+        <v>0.084745763</v>
       </c>
       <c r="H62" s="33" t="n">
         <v>0</v>
@@ -5603,13 +5603,13 @@
         <v>157</v>
       </c>
       <c r="F63" s="33" t="n">
-        <v>0.2922</v>
+        <v>0.02922</v>
       </c>
       <c r="G63" s="33" t="n">
         <v>0</v>
       </c>
       <c r="H63" s="33" t="n">
-        <v>3.50192</v>
+        <v>0.350192</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5629,10 +5629,10 @@
         <v>157</v>
       </c>
       <c r="F64" s="33" t="n">
-        <v>17.839522</v>
+        <v>1.7839522</v>
       </c>
       <c r="G64" s="33" t="n">
-        <v>8.181869</v>
+        <v>0.8181869</v>
       </c>
       <c r="H64" s="33" t="n">
         <v>0</v>
@@ -5658,10 +5658,10 @@
         <v>0</v>
       </c>
       <c r="G65" s="33" t="n">
-        <v>1.01219326</v>
+        <v>0.101219326</v>
       </c>
       <c r="H65" s="33" t="n">
-        <v>1.37142119</v>
+        <v>0.137142119</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,10 +5684,10 @@
         <v>0</v>
       </c>
       <c r="G66" s="33" t="n">
-        <v>0.09568</v>
+        <v>0.009568</v>
       </c>
       <c r="H66" s="33" t="n">
-        <v>0.1196</v>
+        <v>0.01196</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5710,10 +5710,10 @@
         <v>0</v>
       </c>
       <c r="G67" s="33" t="n">
-        <v>0.0844</v>
+        <v>0.00844</v>
       </c>
       <c r="H67" s="33" t="n">
-        <v>0.0211</v>
+        <v>0.00211</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5733,13 +5733,13 @@
         <v>168</v>
       </c>
       <c r="F68" s="33" t="n">
-        <v>0.06559916</v>
+        <v>0.006559916</v>
       </c>
       <c r="G68" s="33" t="n">
-        <v>0.04614793</v>
+        <v>0.004614793</v>
       </c>
       <c r="H68" s="33" t="n">
-        <v>0.01533944</v>
+        <v>0.001533944</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5759,10 +5759,10 @@
         <v>157</v>
       </c>
       <c r="F69" s="33" t="n">
-        <v>0.03535831</v>
+        <v>0.003535831</v>
       </c>
       <c r="G69" s="33" t="n">
-        <v>0.05109999</v>
+        <v>0.005109999</v>
       </c>
       <c r="H69" s="33" t="n">
         <v>0</v>
@@ -5785,7 +5785,7 @@
         <v>168</v>
       </c>
       <c r="F70" s="33" t="n">
-        <v>0.002711</v>
+        <v>0.0002711</v>
       </c>
       <c r="G70" s="33" t="n">
         <v>0</v>
@@ -5811,13 +5811,13 @@
         <v>157</v>
       </c>
       <c r="F71" s="33" t="n">
-        <v>0.07789803</v>
+        <v>0.007789803</v>
       </c>
       <c r="G71" s="33" t="n">
-        <v>0.0036</v>
+        <v>0.00036</v>
       </c>
       <c r="H71" s="33" t="n">
-        <v>0.148</v>
+        <v>0.0148</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5843,7 +5843,7 @@
         <v>0</v>
       </c>
       <c r="H72" s="33" t="n">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5869,7 +5869,7 @@
         <v>0</v>
       </c>
       <c r="H73" s="33" t="n">
-        <v>0.2123802</v>
+        <v>0.02123802</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5892,10 +5892,10 @@
         <v>0</v>
       </c>
       <c r="G74" s="33" t="n">
-        <v>2.72461</v>
+        <v>0.272461</v>
       </c>
       <c r="H74" s="33" t="n">
-        <v>-2.073568</v>
+        <v>-0.2073568</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5915,13 +5915,13 @@
         <v>157</v>
       </c>
       <c r="F75" s="33" t="n">
-        <v>0.02356076</v>
+        <v>0.002356076</v>
       </c>
       <c r="G75" s="33" t="n">
-        <v>0.39835</v>
+        <v>0.039835</v>
       </c>
       <c r="H75" s="33" t="n">
-        <v>0.06333509</v>
+        <v>0.006333509</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5941,7 +5941,7 @@
         <v>157</v>
       </c>
       <c r="F76" s="33" t="n">
-        <v>0.76975</v>
+        <v>0.076975</v>
       </c>
       <c r="G76" s="33" t="n">
         <v>0</v>
@@ -5967,13 +5967,13 @@
         <v>157</v>
       </c>
       <c r="F77" s="33" t="n">
-        <v>1.47217434999999</v>
+        <v>0.147217434999999</v>
       </c>
       <c r="G77" s="33" t="n">
         <v>0</v>
       </c>
       <c r="H77" s="33" t="n">
-        <v>3.83262019000011</v>
+        <v>0.383262019000011</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5982,15 +5982,15 @@
       </c>
       <c r="F78" s="9" t="n">
         <f aca="false">SUM(F5:F77)</f>
-        <v>184.33560404</v>
+        <v>18.433560404</v>
       </c>
       <c r="G78" s="9" t="n">
         <f aca="false">SUM(G5:G77)</f>
-        <v>259.88430681</v>
+        <v>25.988430681</v>
       </c>
       <c r="H78" s="9" t="n">
         <f aca="false">SUM(H5:H77)</f>
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5998,13 +5998,13 @@
         <v>256</v>
       </c>
       <c r="F79" s="13" t="n">
-        <v>184.33560404</v>
+        <v>18.433560404</v>
       </c>
       <c r="G79" s="13" t="n">
-        <v>259.88430681</v>
+        <v>25.988430681</v>
       </c>
       <c r="H79" s="13" t="n">
-        <v>415.52284775</v>
+        <v>41.552284775</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>